<commit_message>
logs account and brand in successful listings
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/successful-run-record.xlsx
+++ b/Full-LC-AUTO/successful-run-record.xlsx
@@ -395,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -411,16 +411,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Beige</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>flipkart</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -430,19 +422,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>shopsy</t>
+          <t>flipkart</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Beige</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>flipkart</t>
+          <t>shopsy</t>
         </is>
       </c>
     </row>
@@ -454,19 +446,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>shopsy</t>
+          <t>flipkart</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Black-baggy</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>flipkart</t>
+          <t>shopsy</t>
         </is>
       </c>
     </row>
@@ -478,19 +470,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>shopsy</t>
+          <t>flipkart</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Black-Plain</t>
+          <t>Black-baggy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>flipkart</t>
+          <t>shopsy</t>
         </is>
       </c>
     </row>
@@ -502,19 +494,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>shopsy</t>
+          <t>flipkart</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>White-Plain</t>
+          <t>Black-Plain</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>flipkart</t>
+          <t>shopsy</t>
         </is>
       </c>
     </row>
@@ -526,19 +518,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>shopsy</t>
+          <t>flipkart</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trouser</t>
+          <t>White-Plain</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>flipkart</t>
+          <t>shopsy</t>
         </is>
       </c>
     </row>
@@ -549,6 +541,18 @@
         </is>
       </c>
       <c r="B13" t="inlineStr">
+        <is>
+          <t>flipkart</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Trouser</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>shopsy</t>
         </is>

</xml_diff>

<commit_message>
better user-inputs for main.py
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/successful-run-record.xlsx
+++ b/Full-LC-AUTO/successful-run-record.xlsx
@@ -395,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -409,10 +409,50 @@
           <t>Surface</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Prabhu</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Seema</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Prabhu</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Seema</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -449,6 +489,11 @@
           <t>flipkart</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>10-STAR</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -545,6 +590,16 @@
           <t>flipkart</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>5-IND</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>5-STAR</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -555,6 +610,11 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>shopsy</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>5-IND</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SCANNIN DIRECTORIES AND LOGGING LISTINGS VIA THAT
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/successful-run-record.xlsx
+++ b/Full-LC-AUTO/successful-run-record.xlsx
@@ -395,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,6 +429,16 @@
           <t>2026-06-19</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -453,6 +463,16 @@
           <t>Seema</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Prabhu</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Seema</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -598,6 +618,11 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>5-STAR</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5-GENZ</t>
         </is>
       </c>
     </row>

</xml_diff>